<commit_message>
Adding new endpoints. For milex roulette
</commit_message>
<xml_diff>
--- a/Files/simulacionAlbum.xlsx
+++ b/Files/simulacionAlbum.xlsx
@@ -8,12 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robertmoreno/Documents/CN/API/API-CN/Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F69AD850-6939-2D4A-AF60-6FF8B1134847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52B80F0A-7C16-0843-B5F2-12B0D54DC0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="17160" xr2:uid="{1AD7F553-B39B-C84C-B751-52623847EF76}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{1AD7F553-B39B-C84C-B751-52623847EF76}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="AR" sheetId="1" r:id="rId1"/>
+    <sheet name="DR" sheetId="2" r:id="rId2"/>
+    <sheet name="ZA" sheetId="3" r:id="rId3"/>
+    <sheet name="HN" sheetId="4" r:id="rId4"/>
+    <sheet name="SV" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="13">
   <si>
     <t>PREMIO</t>
   </si>
@@ -62,9 +66,6 @@
     <t>Stock</t>
   </si>
   <si>
-    <t>RULETA</t>
-  </si>
-  <si>
     <t>Simulación Gloria</t>
   </si>
   <si>
@@ -76,12 +77,15 @@
   <si>
     <t>200 ptos</t>
   </si>
+  <si>
+    <t>JUEGO</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -105,6 +109,13 @@
       <color rgb="FF242424"/>
       <name val="Barlow"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -126,11 +137,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -465,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5615354-CC7E-7946-9B5F-8C27DC9170E8}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
@@ -491,7 +503,7 @@
         <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.25">
@@ -499,7 +511,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2">
         <v>15000</v>
@@ -511,7 +523,7 @@
         <v>99</v>
       </c>
       <c r="F2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.25">
@@ -531,7 +543,7 @@
         <v>99</v>
       </c>
       <c r="F3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.25">
@@ -539,7 +551,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4">
         <v>250</v>
@@ -551,7 +563,7 @@
         <v>99</v>
       </c>
       <c r="F4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="17" x14ac:dyDescent="0.25">
@@ -559,7 +571,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -571,7 +583,7 @@
         <v>99</v>
       </c>
       <c r="F5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="17" x14ac:dyDescent="0.25">
@@ -591,7 +603,7 @@
         <v>99</v>
       </c>
       <c r="F6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.25">
@@ -611,15 +623,615 @@
         <v>99</v>
       </c>
       <c r="F7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.25">
       <c r="B8" s="2"/>
-      <c r="C8">
-        <v>2</v>
-      </c>
       <c r="D8" s="3"/>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B17" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DCE86BE-648C-5144-92FC-490AD2401451}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2">
+        <v>15000</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>98</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>5000</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>98</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4">
+        <v>250</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>98</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <v>100</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>98</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>98</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>98</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EFA61EF-71F3-574F-96B5-7290B7D2025A}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2">
+        <v>15000</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>97</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>5000</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>97</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4">
+        <v>250</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>97</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <v>100</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>97</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>97</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>97</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A501676A-474E-2B47-8A88-503FF7A2AB5F}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2">
+        <v>15000</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>96</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>5000</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>96</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4">
+        <v>250</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>96</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <v>100</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>96</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>96</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>96</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D32FFABA-8453-9C48-B1C0-40EA5075A045}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2">
+        <v>15000</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>95</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>5000</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>95</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4">
+        <v>250</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>95</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <v>100</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>95</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>95</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>95</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>